<commit_message>
Add update workflow refinements
</commit_message>
<xml_diff>
--- a/UPDATE/Projects.xlsx
+++ b/UPDATE/Projects.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="63">
   <si>
     <t>Title</t>
   </si>
@@ -45,7 +45,10 @@
     <t>Premiere</t>
   </si>
   <si>
-    <t>Youtube link</t>
+    <t>Youtube link 1</t>
+  </si>
+  <si>
+    <t>Youtube link 2</t>
   </si>
   <si>
     <t>Circle of Emotions</t>
@@ -115,15 +118,122 @@
   <si>
     <t>https://youtu.be/xQSFbspSqgA?si=XA_n3uNZ0Y3JGbLp</t>
   </si>
+  <si>
+    <t>Irish pub</t>
+  </si>
+  <si>
+    <t>A short musical composition bout the lively culture of Irish pubs</t>
+  </si>
+  <si>
+    <t>October 2020</t>
+  </si>
+  <si>
+    <t>https://youtu.be/CnNnTdbub5I?si=MIdh8dlrQ1TlLgd1</t>
+  </si>
+  <si>
+    <t>Porridge</t>
+  </si>
+  <si>
+    <t>A joyful Avant-Garde composition about the enjoyment of cooking</t>
+  </si>
+  <si>
+    <t>April 2023</t>
+  </si>
+  <si>
+    <t>https://youtu.be/DUywZ53_380?si=fJ2sPwLboOK8K0di</t>
+  </si>
+  <si>
+    <t>War zone</t>
+  </si>
+  <si>
+    <t>Two compositions that faced the complicity of war</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF1155CC"/>
+        <sz val="10.0"/>
+        <u/>
+      </rPr>
+      <t>https://youtu.be/ykamt3_Q9p4?si=joW9bvlp_22IidCg</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF1F1F1F"/>
+        <sz val="10.0"/>
+        <u/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>https://youtu.be/3xfdqgrQJ4g?si=ZMNif1ODHUv04EKE</t>
+  </si>
+  <si>
+    <t>Serious Girl</t>
+  </si>
+  <si>
+    <t>A serious electronic improvisation about a very serious girl</t>
+  </si>
+  <si>
+    <t>Sidney Uzik / Jason Butler / Tara Malone</t>
+  </si>
+  <si>
+    <t>May 2026</t>
+  </si>
+  <si>
+    <t>https://youtu.be/u0rtdx3qxwI?si=F0nB-hEBda3G3Dq_</t>
+  </si>
+  <si>
+    <t>The Owl and the Pussy-Cat</t>
+  </si>
+  <si>
+    <t>Poem by Edward Lear</t>
+  </si>
+  <si>
+    <t>Eran Lavee / Yael Gat / Daniele Pellegrini</t>
+  </si>
+  <si>
+    <t>March 2018</t>
+  </si>
+  <si>
+    <t>https://youtu.be/C5Lh8Fv-zZ8?si=cuU1Yr9sDgutBIR9</t>
+  </si>
+  <si>
+    <t>Berceuse Ensemble</t>
+  </si>
+  <si>
+    <t>An international ensemble presenting a new program of light classical music as part of a diverse and friendly repertoire.</t>
+  </si>
+  <si>
+    <t>During the concert we provide fascinating facts and interesting anecdotes alongside well known classical music, original arrangements and original compositions.</t>
+  </si>
+  <si>
+    <t>December 2022</t>
+  </si>
+  <si>
+    <t>https://youtu.be/pclcCJ6XQ9g?si=OGW7bwwQLN-AQeFh</t>
+  </si>
+  <si>
+    <t>TNEEL</t>
+  </si>
+  <si>
+    <t>Work in progress operetta based on poems by the poet Edward Lear. Combining classical and contemporary music with electronic elements.</t>
+  </si>
+  <si>
+    <t>https://youtu.be/NKpkxzy-Ntg?si=FIoLqjRtfXF65JcN</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="mmmm yyyy"/>
+    <numFmt numFmtId="164" formatCode="mmmm\ yyyy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="15">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -168,26 +278,71 @@
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <u/>
+      <sz val="10.0"/>
+      <color rgb="FF1155CC"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF0F0F0F"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10.0"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF131313"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color theme="1"/>
+      <name val="Amatic SC"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -209,22 +364,34 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="1" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -448,6 +615,7 @@
     <col customWidth="1" min="8" max="8" width="22.13"/>
     <col customWidth="1" min="9" max="9" width="19.38"/>
     <col customWidth="1" min="10" max="10" width="40.38"/>
+    <col customWidth="1" min="11" max="11" width="12.38"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -481,7 +649,9 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2"/>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
@@ -500,32 +670,32 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -546,30 +716,30 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -589,31 +759,31 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="8" t="s">
+      <c r="A4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="B4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>22</v>
+      <c r="C4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I4" s="10">
         <v>46023.0</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -633,16 +803,26 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
+      <c r="A5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>34</v>
+      </c>
       <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
+      <c r="D5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
       <c r="H5" s="12"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="2"/>
+      <c r="I5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>36</v>
+      </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
@@ -661,16 +841,26 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="2"/>
+      <c r="A6" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="12"/>
+      <c r="D6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>40</v>
+      </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -688,18 +878,28 @@
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
+    <row r="7">
+      <c r="A7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="12"/>
+      <c r="D7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>44</v>
+      </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -716,17 +916,31 @@
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="2"/>
+    <row r="8">
+      <c r="A8" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="12"/>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>49</v>
+      </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
@@ -744,17 +958,29 @@
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="2"/>
+    <row r="9">
+      <c r="A9" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="12"/>
+      <c r="D9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>54</v>
+      </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
@@ -772,17 +998,27 @@
       <c r="Y9" s="2"/>
       <c r="Z9" s="2"/>
     </row>
-    <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="2"/>
+    <row r="10">
+      <c r="A10" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="J10" s="13" t="s">
+        <v>59</v>
+      </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
@@ -800,17 +1036,25 @@
       <c r="Y10" s="2"/>
       <c r="Z10" s="2"/>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="2"/>
+    <row r="11">
+      <c r="A11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="12"/>
+      <c r="D11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="13" t="s">
+        <v>62</v>
+      </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
@@ -28525,10 +28769,18 @@
     <hyperlink r:id="rId1" ref="J2"/>
     <hyperlink r:id="rId2" ref="J3"/>
     <hyperlink r:id="rId3" ref="J4"/>
+    <hyperlink r:id="rId4" ref="J5"/>
+    <hyperlink r:id="rId5" ref="J6"/>
+    <hyperlink r:id="rId6" ref="J7"/>
+    <hyperlink r:id="rId7" ref="K7"/>
+    <hyperlink r:id="rId8" ref="J8"/>
+    <hyperlink r:id="rId9" ref="J9"/>
+    <hyperlink r:id="rId10" ref="J10"/>
+    <hyperlink r:id="rId11" ref="J11"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId12"/>
 </worksheet>
 </file>
</xml_diff>